<commit_message>
chore: regenerate all outputs from analysis.py, verify reproducibility
Ran analysis.py from the repo to confirm it reproduces all thesis
figures and tables. Numbers match SA3 reference and thesis exactly.
Removed Sports Analysis 3/ working copy, added to .gitignore.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Analysis/tables/descriptive_stats.xlsx
+++ b/Analysis/tables/descriptive_stats.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Descriptive Statistics" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Means by Outcome" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Region Breakdown" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Region x Outcome Means" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="VIF Diagnostics" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Model C Coefficients" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Model Comparison" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Regional Robustness" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Win Rates by Quartile" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Descriptive Statistics" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Means by Outcome" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Region Breakdown" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Region x Outcome Means" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VIF Diagnostics" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model C Coefficients" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Comparison" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regional Robustness" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Win Rates by Quartile" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>